<commit_message>
fix(git): reinstall autosweep and close sync drift
</commit_message>
<xml_diff>
--- a/项目成员/团队名册_v1.9.xlsx
+++ b/项目成员/团队名册_v1.9.xlsx
@@ -586,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -608,7 +608,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>版本 v1.8 | 2026-05-26 | 项目总监 阿黑</t>
+          <t>版本 v1.9 | 2026-06-12 | 项目总监 阿黑</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>金融线: 用户(创始人) → 阿黑(项目总监) → 腰子(金融负责人) ← 山猫 | 信鸽 | 玉夜 | 流金 | 青山 (专业支撑)</t>
+          <t>金融线: 用户(创始人) → 阿黑(项目总监) → 腰子(金融负责人) ← 山猫 | 信鸽 | 玉夜 | 流金 | 青山 | 砺石(按需方法校准)</t>
         </is>
       </c>
     </row>
@@ -734,7 +734,7 @@
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>投资分析决策核心，协调五位专家，对金融判断质量负责</t>
+          <t>投资分析决策核心，协调六位支撑角色，对金融判断质量负责</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
@@ -939,222 +939,259 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>方法校准官</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>砺石</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>/砺石（按需）</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>方法校准、反证审查、同源证据/因果混淆/结论强度检查 → 支撑腰子的推理链质量</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>告诉腰子这个结论站不站得住</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>.claude/agents/方法校准官-砺石.md</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>.claude/commands/砺石.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>系统架构师</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>情墨</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>/情墨</t>
         </is>
       </c>
-      <c r="D17" s="11" t="inlineStr">
+      <c r="D18" s="11" t="inlineStr">
         <is>
           <t>模块设计、技术选型、API契约、重构决策</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>告诉你系统该怎么搭</t>
         </is>
       </c>
-      <c r="F17" s="11" t="inlineStr">
+      <c r="F18" s="11" t="inlineStr">
         <is>
           <t>.claude/agents/系统架构师-情墨.md</t>
         </is>
       </c>
-      <c r="G17" s="11" t="inlineStr">
+      <c r="G18" s="11" t="inlineStr">
         <is>
           <t>.claude/commands/情墨.md</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>构建工程师(CI)</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>千光</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>/千光</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D19" s="9" t="inlineStr">
         <is>
           <t>自动化流水线、定时调度、代码生成</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E19" s="9" t="inlineStr">
         <is>
           <t>让脚本自己跑起来</t>
         </is>
       </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="F19" s="9" t="inlineStr">
         <is>
           <t>.claude/agents/构建工程师-千光.md</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr">
+      <c r="G19" s="9" t="inlineStr">
         <is>
           <t>.claude/commands/千光.md</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>部署工程师(环境)</t>
         </is>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>红枫</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="C20" s="10" t="inlineStr">
         <is>
           <t>/红枫</t>
         </is>
       </c>
-      <c r="D19" s="11" t="inlineStr">
+      <c r="D20" s="11" t="inlineStr">
         <is>
           <t>环境配置、依赖管理、版本发布、运行监控</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>让系统跑得稳</t>
         </is>
       </c>
-      <c r="F19" s="11" t="inlineStr">
+      <c r="F20" s="11" t="inlineStr">
         <is>
           <t>.claude/agents/部署工程师-红枫.md</t>
         </is>
       </c>
-      <c r="G19" s="11" t="inlineStr">
+      <c r="G20" s="11" t="inlineStr">
         <is>
           <t>.claude/commands/红枫.md</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>质量工程师(测试)</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>新安</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>/新安</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>测试策略、回归验证、变更影响分析</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="E21" s="9" t="inlineStr">
         <is>
           <t>证明改了不会坏</t>
         </is>
       </c>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t>.claude/agents/质量工程师-新安.md</t>
         </is>
       </c>
-      <c r="G20" s="9" t="inlineStr">
+      <c r="G21" s="9" t="inlineStr">
         <is>
           <t>.claude/commands/新安.md</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>代码工匠</t>
         </is>
       </c>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B22" s="10" t="inlineStr">
         <is>
           <t>红结</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="C22" s="10" t="inlineStr">
         <is>
           <t>/红结</t>
         </is>
       </c>
-      <c r="D21" s="11" t="inlineStr">
+      <c r="D22" s="11" t="inlineStr">
         <is>
           <t>PowerShell/Python编码实现、接口落地</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>把设计变成可运行的代码</t>
         </is>
       </c>
-      <c r="F21" s="11" t="inlineStr">
+      <c r="F22" s="11" t="inlineStr">
         <is>
           <t>.claude/agents/代码工匠-红结.md</t>
         </is>
       </c>
-      <c r="G21" s="11" t="inlineStr">
+      <c r="G22" s="11" t="inlineStr">
         <is>
           <t>.claude/commands/红结.md</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>审计官</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>旧影</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>/旧影</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>四级审计(目标对齐/红线执行/成本/技术健康)、问题追踪、修复路线</t>
         </is>
       </c>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="E23" s="9" t="inlineStr">
         <is>
           <t>告诉团队哪里出了问题，怎么修</t>
         </is>
       </c>
-      <c r="F22" s="9" t="inlineStr">
+      <c r="F23" s="9" t="inlineStr">
         <is>
           <t>.claude/agents/审计官-旧影.md</t>
         </is>
       </c>
-      <c r="G22" s="9" t="inlineStr">
+      <c r="G23" s="9" t="inlineStr">
         <is>
           <t>.claude/commands/旧影.md</t>
         </is>
@@ -1179,7 +1216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1194,6 +1231,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -1331,102 +1369,119 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>砺石 — 方法校准官</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>方法校准与反证审查；检查同源证据重复、因果混淆、结论强度过高、隐含假设未说明、反证不足；为腰子提供推理链质量参考；召唤命令为/砺石（按需）</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>不做投资方向判断，不替代腰子裁决；LISHI-SEED规则为L5-seed，未完成15步验证，不得宣称L2或active rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>情墨 — 系统架构师</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>系统模块设计与边界划分、模块间接口契约定义；技术选型评估；数据流设计；重构决策；不写代码，出设计文档和架构图</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C12" s="13" t="inlineStr">
         <is>
           <t>不写代码、不执行部署或运维、不提供金融分析</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>千光 — 构建工程师(CI)</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>CI/CD流水线设计；自动化调度编排；定时任务管理；代码生成方案；不写代码，出流水线设计和调度方案</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>不写代码、不管理服务器环境、不做架构设计</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>红枫 — 部署工程师(环境)</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>环境配置管理；部署策略设计；运行监控方案；备份与恢复；不写代码，出部署方案和环境诊断</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
+      <c r="C14" s="13" t="inlineStr">
         <is>
           <t>不写代码、不设计架构、不构建流水线</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>新安 — 质量工程师(测试)</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>测试策略设计；回归测试用例；变更影响分析；代码规范审查；不写代码，出测试方案和审查报告</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
+      <c r="C15" s="12" t="inlineStr">
         <is>
           <t>不写代码、不修bug、不设计架构或流水线</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>红结 — 代码工匠</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>PowerShell/Python编码实现；接口落地；代码重构执行；按情墨设计和千光流水线规范实现</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C16" s="13" t="inlineStr">
         <is>
           <t>不设计架构、不出测试方案、只按规范写代码</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>旧影 — 审计官</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>独立审计，直接对阿黑负责；四级审计体系(目标对齐/红线执行/成本/技术健康)；发现问题、给出修复指令、追踪修复状态</t>
         </is>
       </c>
-      <c r="C16" s="12" t="inlineStr">
+      <c r="C17" s="12" t="inlineStr">
         <is>
           <t>只审计不执行：发现问题、给出修复指令、追踪修复状态，不自己动手修代码</t>
         </is>
@@ -1446,7 +1501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1460,6 +1515,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -1470,10 +1526,11 @@
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>山猫+信鸽+玉夜+流金+青山 → 腰子(综合判断) → 投资决策</t>
-        </is>
-      </c>
-    </row>
+          <t>山猫+信鸽+玉夜+流金+青山+砺石(按需) → 腰子(综合判断) → 投资决策</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -1537,7 +1594,7 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>腰子 — 六维评分 / 综合判断 / 最终决策 ← 接收四方支撑</t>
+          <t>腰子 — 六维评分 / 综合判断 / 最终决策 ← 接收金融线支撑</t>
         </is>
       </c>
     </row>
@@ -1566,116 +1623,124 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>方法校准</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>协作纪律</t>
         </is>
       </c>
-      <c r="B14" s="16" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="17" t="inlineStr">
+      <c r="B15" s="16" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>腰子是金融线核心</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>所有金融分析任务由腰子主导，协调五位专家，综合各方输出做最终投资判断</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="18" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>所有金融分析任务由腰子主导，协调山猫/信鸽/玉夜/流金/青山/砺石，综合各方输出做最终投资判断</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="inlineStr">
         <is>
           <t>支撑角色向腰子汇报</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
-        <is>
-          <t>山猫/信鸽/玉夜/流金/青山的输出统一给腰子；腰子不在时，阿黑代为接收</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>山猫/信鸽/玉夜/流金/青山/砺石的输出统一给腰子；砺石按需提供方法校准参考</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>分工明确，互不越界</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>腰子不做风控细节，流金不挖因子，青山不看单票，信鸽不做深度解读，山猫不做个股；红结只写代码</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="18" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>金融信息流</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
-        <is>
-          <t>山猫+信鸽+玉夜+流金+青山 → 腰子 → 投资决策</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="17" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>山猫+信鸽+玉夜+流金+青山+砺石(按需) → 腰子 → 投资决策</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>工程信息流</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>情墨设计 → 千光构建 → 红枫部署 → 新安验证 → 红结实现</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="18" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr">
         <is>
           <t>跨团队协作</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>腰子提金融需求 → 阿黑分派工程团队 → 工程团队实施 → 腰子验证金融结果</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="17" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>争议解决</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>金融团队内→腰子判断；工程团队内→阿黑判断；跨线→阿黑协调，用户最终决策</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="18" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="18" t="inlineStr">
         <is>
           <t>红线共守</t>
         </is>
       </c>
-      <c r="B22" s="11" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>所有角色共同遵守规则红线最新版本</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="17" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>审计独立</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>旧影独立于金融线和工程线，直接对阿黑负责；审计结论不受被审计方影响；任何人不得阻止或修改审计发现</t>
         </is>
@@ -1699,7 +1764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25.1" customWidth="1" min="1" max="1"/>
@@ -2359,6 +2424,74 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>砺石方法审查包</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>统一解读/角色解释包/砺石_方法审查包.md</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>砺石方法校准输出模板</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>砺石知识库入口</t>
+        </is>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>00_项目地基/07_知识进化/knowledge/roles/lishi/</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>砺石知识库进化入口与 L5-seed 候选规则池</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>砺石角色定义</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>.claude/agents/方法校准官-砺石.md</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>砺石完整角色定义</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>砺石召唤命令</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>.claude/commands/砺石.md</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>砺石按需召唤入口</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>

</xml_diff>